<commit_message>
Updated the files for SYC, BECF, and BFPaT
</commit_message>
<xml_diff>
--- a/InputData/add-outputs/SCoC/Social Cost of Carbon.xlsx
+++ b/InputData/add-outputs/SCoC/Social Cost of Carbon.xlsx
@@ -1,22 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10211"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Meghan\Dropbox (Energy Innovation)\EPS Versions\eps-1.5.0-us-wipI\InputData\add-outputs\SCoC\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ssy02/Desktop/Indonesia/InputData/add-outputs/SCoC/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97769EB2-12AF-3B43-AB64-CC2F26EE205A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="21075" windowHeight="11820"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="SourceData" sheetId="2" r:id="rId2"/>
     <sheet name="SCoC" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -92,7 +106,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0"/>
@@ -256,17 +270,17 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="8">
-    <cellStyle name="Body: normal cell" xfId="5"/>
-    <cellStyle name="Font: Calibri, 9pt regular" xfId="3"/>
-    <cellStyle name="Footnotes: top row" xfId="7"/>
-    <cellStyle name="Header: bottom row" xfId="4"/>
+    <cellStyle name="Body: normal cell" xfId="5" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
+    <cellStyle name="Font: Calibri, 9pt regular" xfId="3" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="Footnotes: top row" xfId="7" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="Header: bottom row" xfId="4" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Parent row" xfId="6"/>
-    <cellStyle name="Table title" xfId="2"/>
+    <cellStyle name="Parent row" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="Table title" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -282,9 +296,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -322,9 +336,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -359,7 +373,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -394,7 +408,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -567,19 +581,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="97.140625" customWidth="1"/>
+    <col min="2" max="2" width="97.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -587,68 +601,68 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B4" s="2">
         <v>2015</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B6" s="3" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:2" s="13" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="13" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="13" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" s="13">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17">
         <v>1.109</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="13" t="s">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>15</v>
       </c>
     </row>
@@ -659,15 +673,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:K64"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" customWidth="1"/>
-    <col min="7" max="7" width="13.85546875" customWidth="1"/>
+    <col min="1" max="1" width="13.5" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" s="8" t="s">
         <v>8</v>
       </c>
@@ -683,7 +697,7 @@
       <c r="J1" s="11"/>
       <c r="K1" s="11"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>3</v>
       </c>
@@ -715,7 +729,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>5</v>
       </c>
@@ -747,8 +761,8 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" s="13">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4">
         <v>2010</v>
       </c>
       <c r="B4" s="7">
@@ -784,8 +798,8 @@
         <v>9.5373999999999999E-5</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="13">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5">
         <v>2011</v>
       </c>
       <c r="B5" s="7">
@@ -821,8 +835,8 @@
         <v>9.9810000000000008E-5</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" s="13">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A6">
         <v>2012</v>
       </c>
       <c r="B6" s="7">
@@ -858,8 +872,8 @@
         <v>1.03137E-4</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="13">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A7">
         <v>2013</v>
       </c>
       <c r="B7" s="7">
@@ -895,8 +909,8 @@
         <v>1.0757299999999999E-4</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="13">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8">
         <v>2014</v>
       </c>
       <c r="B8" s="7">
@@ -932,8 +946,8 @@
         <v>1.12009E-4</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A9" s="13">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9">
         <v>2015</v>
       </c>
       <c r="B9" s="7">
@@ -969,8 +983,8 @@
         <v>1.1644499999999999E-4</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A10" s="13">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10">
         <v>2016</v>
       </c>
       <c r="B10" s="7">
@@ -1006,8 +1020,8 @@
         <v>1.1977199999999999E-4</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A11" s="13">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A11">
         <v>2017</v>
       </c>
       <c r="B11" s="7">
@@ -1043,8 +1057,8 @@
         <v>1.24208E-4</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A12" s="13">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A12">
         <v>2018</v>
       </c>
       <c r="B12" s="7">
@@ -1080,8 +1094,8 @@
         <v>1.28644E-4</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A13" s="13">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A13">
         <v>2019</v>
       </c>
       <c r="B13" s="7">
@@ -1117,8 +1131,8 @@
         <v>1.3307999999999999E-4</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="13">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A14">
         <v>2020</v>
       </c>
       <c r="B14" s="7">
@@ -1154,8 +1168,8 @@
         <v>1.3640700000000001E-4</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A15" s="13">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15">
         <v>2021</v>
       </c>
       <c r="B15" s="7">
@@ -1191,8 +1205,8 @@
         <v>1.39734E-4</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A16" s="13">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16">
         <v>2022</v>
       </c>
       <c r="B16" s="7">
@@ -1228,8 +1242,8 @@
         <v>1.4306100000000002E-4</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A17" s="13">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A17">
         <v>2023</v>
       </c>
       <c r="B17" s="7">
@@ -1265,8 +1279,8 @@
         <v>1.4638800000000001E-4</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A18" s="13">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A18">
         <v>2024</v>
       </c>
       <c r="B18" s="7">
@@ -1302,8 +1316,8 @@
         <v>1.49715E-4</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A19" s="13">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A19">
         <v>2025</v>
       </c>
       <c r="B19" s="7">
@@ -1339,8 +1353,8 @@
         <v>1.5304199999999999E-4</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A20" s="13">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A20">
         <v>2026</v>
       </c>
       <c r="B20" s="7">
@@ -1376,8 +1390,8 @@
         <v>1.5636900000000001E-4</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A21" s="13">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A21">
         <v>2027</v>
       </c>
       <c r="B21" s="7">
@@ -1413,8 +1427,8 @@
         <v>1.5858699999999999E-4</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A22" s="13">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A22">
         <v>2028</v>
       </c>
       <c r="B22" s="7">
@@ -1450,8 +1464,8 @@
         <v>1.6191399999999998E-4</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A23" s="13">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A23">
         <v>2029</v>
       </c>
       <c r="B23" s="7">
@@ -1487,8 +1501,8 @@
         <v>1.65241E-4</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A24" s="13">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A24">
         <v>2030</v>
       </c>
       <c r="B24" s="7">
@@ -1524,8 +1538,8 @@
         <v>1.6856799999999999E-4</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A25" s="13">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A25">
         <v>2031</v>
       </c>
       <c r="B25" s="7">
@@ -1561,8 +1575,8 @@
         <v>1.7189500000000001E-4</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A26" s="13">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A26">
         <v>2032</v>
       </c>
       <c r="B26" s="7">
@@ -1598,8 +1612,8 @@
         <v>1.75222E-4</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A27" s="13">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A27">
         <v>2033</v>
       </c>
       <c r="B27" s="7">
@@ -1635,8 +1649,8 @@
         <v>1.7854900000000001E-4</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="13">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A28">
         <v>2034</v>
       </c>
       <c r="B28" s="7">
@@ -1672,8 +1686,8 @@
         <v>1.81876E-4</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A29" s="13">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A29">
         <v>2035</v>
       </c>
       <c r="B29" s="7">
@@ -1709,8 +1723,8 @@
         <v>1.86312E-4</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A30" s="13">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A30">
         <v>2036</v>
       </c>
       <c r="B30" s="7">
@@ -1746,8 +1760,8 @@
         <v>1.8963900000000002E-4</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" s="13">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A31">
         <v>2037</v>
       </c>
       <c r="B31" s="7">
@@ -1783,8 +1797,8 @@
         <v>1.9296600000000001E-4</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" s="13">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A32">
         <v>2038</v>
       </c>
       <c r="B32" s="7">
@@ -1820,8 +1834,8 @@
         <v>1.96293E-4</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A33" s="13">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A33">
         <v>2039</v>
       </c>
       <c r="B33" s="7">
@@ -1857,8 +1871,8 @@
         <v>1.9962000000000002E-4</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" s="13">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A34">
         <v>2040</v>
       </c>
       <c r="B34" s="7">
@@ -1894,8 +1908,8 @@
         <v>2.0294700000000001E-4</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" s="13">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A35">
         <v>2041</v>
       </c>
       <c r="B35" s="7">
@@ -1931,8 +1945,8 @@
         <v>2.06274E-4</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" s="13">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A36">
         <v>2042</v>
       </c>
       <c r="B36" s="7">
@@ -1968,8 +1982,8 @@
         <v>2.0960099999999999E-4</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A37" s="13">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A37">
         <v>2043</v>
       </c>
       <c r="B37" s="7">
@@ -2005,8 +2019,8 @@
         <v>2.1292800000000001E-4</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A38" s="13">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A38">
         <v>2044</v>
       </c>
       <c r="B38" s="7">
@@ -2042,8 +2056,8 @@
         <v>2.1514599999999999E-4</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A39" s="13">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A39">
         <v>2045</v>
       </c>
       <c r="B39" s="7">
@@ -2079,8 +2093,8 @@
         <v>2.1847299999999998E-4</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A40" s="13">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A40">
         <v>2046</v>
       </c>
       <c r="B40" s="7">
@@ -2116,8 +2130,8 @@
         <v>2.2180000000000002E-4</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A41" s="13">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A41">
         <v>2047</v>
       </c>
       <c r="B41" s="7">
@@ -2153,8 +2167,8 @@
         <v>2.2512700000000001E-4</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A42" s="13">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A42">
         <v>2048</v>
       </c>
       <c r="B42" s="7">
@@ -2190,8 +2204,8 @@
         <v>2.2845400000000001E-4</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A43" s="13">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A43">
         <v>2049</v>
       </c>
       <c r="B43" s="7">
@@ -2227,8 +2241,8 @@
         <v>2.31781E-4</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A44" s="13">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A44">
         <v>2050</v>
       </c>
       <c r="B44" s="7">
@@ -2262,6 +2276,806 @@
       <c r="K44" s="12">
         <f>E44*(About!$A$17)/10^6</f>
         <v>2.3510800000000001E-4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A45" s="13">
+        <v>2051</v>
+      </c>
+      <c r="B45">
+        <f>_xlfn.FORECAST.LINEAR(A45,B4:B44,A4:A44)</f>
+        <v>25.146341463414615</v>
+      </c>
+      <c r="C45">
+        <f t="shared" ref="C45:E45" si="1">_xlfn.FORECAST.LINEAR(B45,C4:C44,B4:B44)</f>
+        <v>69.238104101362381</v>
+      </c>
+      <c r="D45">
+        <f t="shared" si="1"/>
+        <v>95.349352804211989</v>
+      </c>
+      <c r="E45">
+        <f t="shared" si="1"/>
+        <v>214.48217386448064</v>
+      </c>
+      <c r="G45" s="1">
+        <v>2051</v>
+      </c>
+      <c r="H45" s="12">
+        <f>B45*(About!$A$17)/10^6</f>
+        <v>2.788729268292681E-5</v>
+      </c>
+      <c r="I45" s="12">
+        <f>C45*(About!$A$17)/10^6</f>
+        <v>7.6785057448410887E-5</v>
+      </c>
+      <c r="J45" s="12">
+        <f>D45*(About!$A$17)/10^6</f>
+        <v>1.0574243225987109E-4</v>
+      </c>
+      <c r="K45" s="12">
+        <f>E45*(About!$A$17)/10^6</f>
+        <v>2.3786073081570903E-4</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A46" s="13">
+        <v>2052</v>
+      </c>
+      <c r="B46">
+        <f t="shared" ref="B46:B64" si="2">_xlfn.FORECAST.LINEAR(A46,B5:B45,A5:A45)</f>
+        <v>25.625252825699022</v>
+      </c>
+      <c r="C46">
+        <f t="shared" ref="C46:C64" si="3">_xlfn.FORECAST.LINEAR(B46,C5:C45,B5:B45)</f>
+        <v>70.13507116364471</v>
+      </c>
+      <c r="D46">
+        <f t="shared" ref="D46:D64" si="4">_xlfn.FORECAST.LINEAR(C46,D5:D45,C5:C45)</f>
+        <v>96.430906777724857</v>
+      </c>
+      <c r="E46">
+        <f t="shared" ref="E46:E64" si="5">_xlfn.FORECAST.LINEAR(D46,E5:E45,D5:D45)</f>
+        <v>217.39445741754284</v>
+      </c>
+      <c r="G46" s="1">
+        <v>2052</v>
+      </c>
+      <c r="H46" s="12">
+        <f>B46*(About!$A$17)/10^6</f>
+        <v>2.8418405383700215E-5</v>
+      </c>
+      <c r="I46" s="12">
+        <f>C46*(About!$A$17)/10^6</f>
+        <v>7.7779793920481984E-5</v>
+      </c>
+      <c r="J46" s="12">
+        <f>D46*(About!$A$17)/10^6</f>
+        <v>1.0694187561649686E-4</v>
+      </c>
+      <c r="K46" s="12">
+        <f>E46*(About!$A$17)/10^6</f>
+        <v>2.4109045327605499E-4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A47" s="13">
+        <v>2053</v>
+      </c>
+      <c r="B47">
+        <f t="shared" si="2"/>
+        <v>26.147912827730352</v>
+      </c>
+      <c r="C47">
+        <f t="shared" si="3"/>
+        <v>71.094552833435401</v>
+      </c>
+      <c r="D47">
+        <f t="shared" si="4"/>
+        <v>97.578921591079023</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="5"/>
+        <v>220.5361315635831</v>
+      </c>
+      <c r="G47" s="1">
+        <v>2053</v>
+      </c>
+      <c r="H47" s="12">
+        <f>B47*(About!$A$17)/10^6</f>
+        <v>2.8998035325952957E-5</v>
+      </c>
+      <c r="I47" s="12">
+        <f>C47*(About!$A$17)/10^6</f>
+        <v>7.8843859092279862E-5</v>
+      </c>
+      <c r="J47" s="12">
+        <f>D47*(About!$A$17)/10^6</f>
+        <v>1.0821502404450664E-4</v>
+      </c>
+      <c r="K47" s="12">
+        <f>E47*(About!$A$17)/10^6</f>
+        <v>2.4457456990401364E-4</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A48" s="13">
+        <v>2054</v>
+      </c>
+      <c r="B48">
+        <f t="shared" si="2"/>
+        <v>26.668057026938982</v>
+      </c>
+      <c r="C48">
+        <f t="shared" si="3"/>
+        <v>72.03371282242847</v>
+      </c>
+      <c r="D48">
+        <f t="shared" si="4"/>
+        <v>98.747695403285846</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="5"/>
+        <v>223.59618914930002</v>
+      </c>
+      <c r="G48" s="1">
+        <v>2054</v>
+      </c>
+      <c r="H48" s="12">
+        <f>B48*(About!$A$17)/10^6</f>
+        <v>2.9574875242875329E-5</v>
+      </c>
+      <c r="I48" s="12">
+        <f>C48*(About!$A$17)/10^6</f>
+        <v>7.9885387520073171E-5</v>
+      </c>
+      <c r="J48" s="12">
+        <f>D48*(About!$A$17)/10^6</f>
+        <v>1.09511194202244E-4</v>
+      </c>
+      <c r="K48" s="12">
+        <f>E48*(About!$A$17)/10^6</f>
+        <v>2.4796817376657372E-4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A49" s="13">
+        <v>2055</v>
+      </c>
+      <c r="B49">
+        <f t="shared" si="2"/>
+        <v>27.183527808407916</v>
+      </c>
+      <c r="C49">
+        <f t="shared" si="3"/>
+        <v>72.952885528979863</v>
+      </c>
+      <c r="D49">
+        <f t="shared" si="4"/>
+        <v>99.890782879628816</v>
+      </c>
+      <c r="E49">
+        <f t="shared" si="5"/>
+        <v>226.61308438710225</v>
+      </c>
+      <c r="G49" s="1">
+        <v>2055</v>
+      </c>
+      <c r="H49" s="12">
+        <f>B49*(About!$A$17)/10^6</f>
+        <v>3.0146532339524376E-5</v>
+      </c>
+      <c r="I49" s="12">
+        <f>C49*(About!$A$17)/10^6</f>
+        <v>8.0904750051638674E-5</v>
+      </c>
+      <c r="J49" s="12">
+        <f>D49*(About!$A$17)/10^6</f>
+        <v>1.1077887821350835E-4</v>
+      </c>
+      <c r="K49" s="12">
+        <f>E49*(About!$A$17)/10^6</f>
+        <v>2.5131391058529637E-4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A50" s="13">
+        <v>2056</v>
+      </c>
+      <c r="B50">
+        <f t="shared" si="2"/>
+        <v>27.691966262360665</v>
+      </c>
+      <c r="C50">
+        <f t="shared" si="3"/>
+        <v>73.852703071535274</v>
+      </c>
+      <c r="D50">
+        <f t="shared" si="4"/>
+        <v>101.00747132573326</v>
+      </c>
+      <c r="E50">
+        <f t="shared" si="5"/>
+        <v>229.59517810114383</v>
+      </c>
+      <c r="G50" s="1">
+        <v>2056</v>
+      </c>
+      <c r="H50" s="12">
+        <f>B50*(About!$A$17)/10^6</f>
+        <v>3.0710390584957974E-5</v>
+      </c>
+      <c r="I50" s="12">
+        <f>C50*(About!$A$17)/10^6</f>
+        <v>8.1902647706332622E-5</v>
+      </c>
+      <c r="J50" s="12">
+        <f>D50*(About!$A$17)/10^6</f>
+        <v>1.1201728570023819E-4</v>
+      </c>
+      <c r="K50" s="12">
+        <f>E50*(About!$A$17)/10^6</f>
+        <v>2.5462105251416848E-4</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A51" s="13">
+        <v>2057</v>
+      </c>
+      <c r="B51">
+        <f t="shared" si="2"/>
+        <v>28.190800439351278</v>
+      </c>
+      <c r="C51">
+        <f t="shared" si="3"/>
+        <v>74.734209944863807</v>
+      </c>
+      <c r="D51">
+        <f t="shared" si="4"/>
+        <v>102.0974826017151</v>
+      </c>
+      <c r="E51">
+        <f t="shared" si="5"/>
+        <v>232.55270026102519</v>
+      </c>
+      <c r="G51" s="1">
+        <v>2057</v>
+      </c>
+      <c r="H51" s="12">
+        <f>B51*(About!$A$17)/10^6</f>
+        <v>3.1263597687240563E-5</v>
+      </c>
+      <c r="I51" s="12">
+        <f>C51*(About!$A$17)/10^6</f>
+        <v>8.2880238828853957E-5</v>
+      </c>
+      <c r="J51" s="12">
+        <f>D51*(About!$A$17)/10^6</f>
+        <v>1.1322610820530204E-4</v>
+      </c>
+      <c r="K51" s="12">
+        <f>E51*(About!$A$17)/10^6</f>
+        <v>2.5790094458947693E-4</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A52" s="13">
+        <v>2058</v>
+      </c>
+      <c r="B52">
+        <f t="shared" si="2"/>
+        <v>28.677233196064094</v>
+      </c>
+      <c r="C52">
+        <f t="shared" si="3"/>
+        <v>75.643060138832652</v>
+      </c>
+      <c r="D52">
+        <f t="shared" si="4"/>
+        <v>103.15035609891419</v>
+      </c>
+      <c r="E52">
+        <f t="shared" si="5"/>
+        <v>235.41407090604022</v>
+      </c>
+      <c r="G52" s="1">
+        <v>2058</v>
+      </c>
+      <c r="H52" s="12">
+        <f>B52*(About!$A$17)/10^6</f>
+        <v>3.1803051614435077E-5</v>
+      </c>
+      <c r="I52" s="12">
+        <f>C52*(About!$A$17)/10^6</f>
+        <v>8.3888153693965412E-5</v>
+      </c>
+      <c r="J52" s="12">
+        <f>D52*(About!$A$17)/10^6</f>
+        <v>1.1439374491369583E-4</v>
+      </c>
+      <c r="K52" s="12">
+        <f>E52*(About!$A$17)/10^6</f>
+        <v>2.6107420463479861E-4</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A53" s="13">
+        <v>2059</v>
+      </c>
+      <c r="B53">
+        <f t="shared" si="2"/>
+        <v>29.148229634751146</v>
+      </c>
+      <c r="C53">
+        <f t="shared" si="3"/>
+        <v>76.548404105479392</v>
+      </c>
+      <c r="D53">
+        <f t="shared" si="4"/>
+        <v>104.2329373036404</v>
+      </c>
+      <c r="E53">
+        <f t="shared" si="5"/>
+        <v>238.27650834249363</v>
+      </c>
+      <c r="G53" s="1">
+        <v>2059</v>
+      </c>
+      <c r="H53" s="12">
+        <f>B53*(About!$A$17)/10^6</f>
+        <v>3.2325386664939019E-5</v>
+      </c>
+      <c r="I53" s="12">
+        <f>C53*(About!$A$17)/10^6</f>
+        <v>8.4892180152976656E-5</v>
+      </c>
+      <c r="J53" s="12">
+        <f>D53*(About!$A$17)/10^6</f>
+        <v>1.1559432746973719E-4</v>
+      </c>
+      <c r="K53" s="12">
+        <f>E53*(About!$A$17)/10^6</f>
+        <v>2.6424864775182545E-4</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A54" s="13">
+        <v>2060</v>
+      </c>
+      <c r="B54">
+        <f t="shared" si="2"/>
+        <v>29.652943165519559</v>
+      </c>
+      <c r="C54">
+        <f t="shared" si="3"/>
+        <v>77.476975832843692</v>
+      </c>
+      <c r="D54">
+        <f t="shared" si="4"/>
+        <v>105.33230512736525</v>
+      </c>
+      <c r="E54">
+        <f t="shared" si="5"/>
+        <v>241.23049554271282</v>
+      </c>
+      <c r="G54" s="1">
+        <v>2060</v>
+      </c>
+      <c r="H54" s="12">
+        <f>B54*(About!$A$17)/10^6</f>
+        <v>3.2885113970561193E-5</v>
+      </c>
+      <c r="I54" s="12">
+        <f>C54*(About!$A$17)/10^6</f>
+        <v>8.5921966198623651E-5</v>
+      </c>
+      <c r="J54" s="12">
+        <f>D54*(About!$A$17)/10^6</f>
+        <v>1.1681352638624806E-4</v>
+      </c>
+      <c r="K54" s="12">
+        <f>E54*(About!$A$17)/10^6</f>
+        <v>2.6752461955686853E-4</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A55" s="13">
+        <v>2061</v>
+      </c>
+      <c r="B55">
+        <f t="shared" si="2"/>
+        <v>30.144159615260378</v>
+      </c>
+      <c r="C55">
+        <f t="shared" si="3"/>
+        <v>78.402413372298327</v>
+      </c>
+      <c r="D55">
+        <f t="shared" si="4"/>
+        <v>106.41524484943689</v>
+      </c>
+      <c r="E55">
+        <f t="shared" si="5"/>
+        <v>244.19523744853441</v>
+      </c>
+      <c r="G55" s="1">
+        <v>2061</v>
+      </c>
+      <c r="H55" s="12">
+        <f>B55*(About!$A$17)/10^6</f>
+        <v>3.3429873013323756E-5</v>
+      </c>
+      <c r="I55" s="12">
+        <f>C55*(About!$A$17)/10^6</f>
+        <v>8.6948276429878846E-5</v>
+      </c>
+      <c r="J55" s="12">
+        <f>D55*(About!$A$17)/10^6</f>
+        <v>1.1801450653802551E-4</v>
+      </c>
+      <c r="K55" s="12">
+        <f>E55*(About!$A$17)/10^6</f>
+        <v>2.7081251833042469E-4</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A56" s="13">
+        <v>2062</v>
+      </c>
+      <c r="B56">
+        <f t="shared" si="2"/>
+        <v>30.618715682663037</v>
+      </c>
+      <c r="C56">
+        <f t="shared" si="3"/>
+        <v>79.329450600374969</v>
+      </c>
+      <c r="D56">
+        <f t="shared" si="4"/>
+        <v>107.48590343683686</v>
+      </c>
+      <c r="E56">
+        <f t="shared" si="5"/>
+        <v>247.1406830162536</v>
+      </c>
+      <c r="G56" s="1">
+        <v>2062</v>
+      </c>
+      <c r="H56" s="12">
+        <f>B56*(About!$A$17)/10^6</f>
+        <v>3.3956155692073307E-5</v>
+      </c>
+      <c r="I56" s="12">
+        <f>C56*(About!$A$17)/10^6</f>
+        <v>8.7976360715815845E-5</v>
+      </c>
+      <c r="J56" s="12">
+        <f>D56*(About!$A$17)/10^6</f>
+        <v>1.1920186691145209E-4</v>
+      </c>
+      <c r="K56" s="12">
+        <f>E56*(About!$A$17)/10^6</f>
+        <v>2.7407901746502524E-4</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A57" s="13">
+        <v>2063</v>
+      </c>
+      <c r="B57">
+        <f t="shared" si="2"/>
+        <v>31.073188831219682</v>
+      </c>
+      <c r="C57">
+        <f t="shared" si="3"/>
+        <v>80.212540124961123</v>
+      </c>
+      <c r="D57">
+        <f t="shared" si="4"/>
+        <v>108.54736921772884</v>
+      </c>
+      <c r="E57">
+        <f t="shared" si="5"/>
+        <v>250.07784597732541</v>
+      </c>
+      <c r="G57" s="1">
+        <v>2063</v>
+      </c>
+      <c r="H57" s="12">
+        <f>B57*(About!$A$17)/10^6</f>
+        <v>3.4460166413822628E-5</v>
+      </c>
+      <c r="I57" s="12">
+        <f>C57*(About!$A$17)/10^6</f>
+        <v>8.8955706998581889E-5</v>
+      </c>
+      <c r="J57" s="12">
+        <f>D57*(About!$A$17)/10^6</f>
+        <v>1.2037903246246129E-4</v>
+      </c>
+      <c r="K57" s="12">
+        <f>E57*(About!$A$17)/10^6</f>
+        <v>2.7733633118885389E-4</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A58" s="13">
+        <v>2064</v>
+      </c>
+      <c r="B58">
+        <f t="shared" si="2"/>
+        <v>31.556322595430856</v>
+      </c>
+      <c r="C58">
+        <f t="shared" si="3"/>
+        <v>81.104664853025639</v>
+      </c>
+      <c r="D58">
+        <f t="shared" si="4"/>
+        <v>109.61029818927253</v>
+      </c>
+      <c r="E58">
+        <f t="shared" si="5"/>
+        <v>253.03875751639066</v>
+      </c>
+      <c r="G58" s="1">
+        <v>2064</v>
+      </c>
+      <c r="H58" s="12">
+        <f>B58*(About!$A$17)/10^6</f>
+        <v>3.4995961758332817E-5</v>
+      </c>
+      <c r="I58" s="12">
+        <f>C58*(About!$A$17)/10^6</f>
+        <v>8.994507332200543E-5</v>
+      </c>
+      <c r="J58" s="12">
+        <f>D58*(About!$A$17)/10^6</f>
+        <v>1.2155782069190323E-4</v>
+      </c>
+      <c r="K58" s="12">
+        <f>E58*(About!$A$17)/10^6</f>
+        <v>2.8061998208567723E-4</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A59" s="13">
+        <v>2065</v>
+      </c>
+      <c r="B59">
+        <f t="shared" si="2"/>
+        <v>32.02046993847523</v>
+      </c>
+      <c r="C59">
+        <f t="shared" si="3"/>
+        <v>81.993808430489082</v>
+      </c>
+      <c r="D59">
+        <f t="shared" si="4"/>
+        <v>110.65877845537133</v>
+      </c>
+      <c r="E59">
+        <f t="shared" si="5"/>
+        <v>255.98294586664764</v>
+      </c>
+      <c r="G59" s="1">
+        <v>2065</v>
+      </c>
+      <c r="H59" s="12">
+        <f>B59*(About!$A$17)/10^6</f>
+        <v>3.551070116176903E-5</v>
+      </c>
+      <c r="I59" s="12">
+        <f>C59*(About!$A$17)/10^6</f>
+        <v>9.0931133549412388E-5</v>
+      </c>
+      <c r="J59" s="12">
+        <f>D59*(About!$A$17)/10^6</f>
+        <v>1.2272058530700679E-4</v>
+      </c>
+      <c r="K59" s="12">
+        <f>E59*(About!$A$17)/10^6</f>
+        <v>2.8388508696611221E-4</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A60" s="13">
+        <v>2066</v>
+      </c>
+      <c r="B60">
+        <f t="shared" si="2"/>
+        <v>32.462010964028309</v>
+      </c>
+      <c r="C60">
+        <f t="shared" si="3"/>
+        <v>82.886534939177665</v>
+      </c>
+      <c r="D60">
+        <f t="shared" si="4"/>
+        <v>111.69903314569318</v>
+      </c>
+      <c r="E60">
+        <f t="shared" si="5"/>
+        <v>258.93090509191018</v>
+      </c>
+      <c r="G60" s="1">
+        <v>2066</v>
+      </c>
+      <c r="H60" s="12">
+        <f>B60*(About!$A$17)/10^6</f>
+        <v>3.60003701591074E-5</v>
+      </c>
+      <c r="I60" s="12">
+        <f>C60*(About!$A$17)/10^6</f>
+        <v>9.1921167247548021E-5</v>
+      </c>
+      <c r="J60" s="12">
+        <f>D60*(About!$A$17)/10^6</f>
+        <v>1.2387422775857375E-4</v>
+      </c>
+      <c r="K60" s="12">
+        <f>E60*(About!$A$17)/10^6</f>
+        <v>2.8715437374692839E-4</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A61" s="13">
+        <v>2067</v>
+      </c>
+      <c r="B61">
+        <f t="shared" si="2"/>
+        <v>32.929481102055661</v>
+      </c>
+      <c r="C61">
+        <f t="shared" si="3"/>
+        <v>83.783576788626718</v>
+      </c>
+      <c r="D61">
+        <f t="shared" si="4"/>
+        <v>112.78236009309623</v>
+      </c>
+      <c r="E61">
+        <f t="shared" si="5"/>
+        <v>261.87921134320777</v>
+      </c>
+      <c r="G61" s="1">
+        <v>2067</v>
+      </c>
+      <c r="H61" s="12">
+        <f>B61*(About!$A$17)/10^6</f>
+        <v>3.6518794542179729E-5</v>
+      </c>
+      <c r="I61" s="12">
+        <f>C61*(About!$A$17)/10^6</f>
+        <v>9.2915986658587027E-5</v>
+      </c>
+      <c r="J61" s="12">
+        <f>D61*(About!$A$17)/10^6</f>
+        <v>1.2507563734324371E-4</v>
+      </c>
+      <c r="K61" s="12">
+        <f>E61*(About!$A$17)/10^6</f>
+        <v>2.9042404537961745E-4</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A62" s="13">
+        <v>2068</v>
+      </c>
+      <c r="B62">
+        <f t="shared" si="2"/>
+        <v>33.375014140265989</v>
+      </c>
+      <c r="C62">
+        <f t="shared" si="3"/>
+        <v>84.685234069305068</v>
+      </c>
+      <c r="D62">
+        <f t="shared" si="4"/>
+        <v>113.86348765161344</v>
+      </c>
+      <c r="E62">
+        <f t="shared" si="5"/>
+        <v>264.82845027887151</v>
+      </c>
+      <c r="G62" s="1">
+        <v>2068</v>
+      </c>
+      <c r="H62" s="12">
+        <f>B62*(About!$A$17)/10^6</f>
+        <v>3.7012890681554977E-5</v>
+      </c>
+      <c r="I62" s="12">
+        <f>C62*(About!$A$17)/10^6</f>
+        <v>9.3915924582859314E-5</v>
+      </c>
+      <c r="J62" s="12">
+        <f>D62*(About!$A$17)/10^6</f>
+        <v>1.2627460780563932E-4</v>
+      </c>
+      <c r="K62" s="12">
+        <f>E62*(About!$A$17)/10^6</f>
+        <v>2.9369475135926847E-4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A63" s="13">
+        <v>2069</v>
+      </c>
+      <c r="B63">
+        <f t="shared" si="2"/>
+        <v>33.847198641586942</v>
+      </c>
+      <c r="C63">
+        <f t="shared" si="3"/>
+        <v>85.593399144233587</v>
+      </c>
+      <c r="D63">
+        <f t="shared" si="4"/>
+        <v>114.94333224179115</v>
+      </c>
+      <c r="E63">
+        <f t="shared" si="5"/>
+        <v>267.73141128138741</v>
+      </c>
+      <c r="G63" s="1">
+        <v>2069</v>
+      </c>
+      <c r="H63" s="12">
+        <f>B63*(About!$A$17)/10^6</f>
+        <v>3.7536543293519921E-5</v>
+      </c>
+      <c r="I63" s="12">
+        <f>C63*(About!$A$17)/10^6</f>
+        <v>9.4923079650955047E-5</v>
+      </c>
+      <c r="J63" s="12">
+        <f>D63*(About!$A$17)/10^6</f>
+        <v>1.2747215545614638E-4</v>
+      </c>
+      <c r="K63" s="12">
+        <f>E63*(About!$A$17)/10^6</f>
+        <v>2.9691413511105864E-4</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A64" s="13">
+        <v>2070</v>
+      </c>
+      <c r="B64">
+        <f t="shared" si="2"/>
+        <v>34.298224262035887</v>
+      </c>
+      <c r="C64">
+        <f t="shared" si="3"/>
+        <v>86.507342744777162</v>
+      </c>
+      <c r="D64">
+        <f t="shared" si="4"/>
+        <v>116.01962841052305</v>
+      </c>
+      <c r="E64">
+        <f t="shared" si="5"/>
+        <v>270.62642897051728</v>
+      </c>
+      <c r="G64" s="1">
+        <v>2070</v>
+      </c>
+      <c r="H64" s="12">
+        <f>B64*(About!$A$17)/10^6</f>
+        <v>3.8036730706597802E-5</v>
+      </c>
+      <c r="I64" s="12">
+        <f>C64*(About!$A$17)/10^6</f>
+        <v>9.5936643103957875E-5</v>
+      </c>
+      <c r="J64" s="12">
+        <f>D64*(About!$A$17)/10^6</f>
+        <v>1.2866576790727005E-4</v>
+      </c>
+      <c r="K64" s="12">
+        <f>E64*(About!$A$17)/10^6</f>
+        <v>3.0012470972830366E-4</v>
       </c>
     </row>
   </sheetData>
@@ -2270,17 +3084,17 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:B42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B62"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="24.140625" customWidth="1"/>
+    <col min="2" max="2" width="24.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>4</v>
       </c>
@@ -2288,7 +3102,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2">
         <f>SourceData!G4</f>
         <v>2010</v>
@@ -2298,7 +3112,7 @@
         <v>3.4378999999999997E-5</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3">
         <f>SourceData!G5</f>
         <v>2011</v>
@@ -2308,7 +3122,7 @@
         <v>3.5487999999999996E-5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4">
         <f>SourceData!G6</f>
         <v>2012</v>
@@ -2318,7 +3132,7 @@
         <v>3.6597000000000002E-5</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5">
         <f>SourceData!G7</f>
         <v>2013</v>
@@ -2328,7 +3142,7 @@
         <v>3.7706000000000001E-5</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6">
         <f>SourceData!G8</f>
         <v>2014</v>
@@ -2338,7 +3152,7 @@
         <v>3.8815E-5</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7">
         <f>SourceData!G9</f>
         <v>2015</v>
@@ -2348,7 +3162,7 @@
         <v>3.9923999999999999E-5</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8">
         <f>SourceData!G10</f>
         <v>2016</v>
@@ -2358,7 +3172,7 @@
         <v>4.2141999999999997E-5</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9">
         <f>SourceData!G11</f>
         <v>2017</v>
@@ -2368,7 +3182,7 @@
         <v>4.3250999999999996E-5</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10">
         <f>SourceData!G12</f>
         <v>2018</v>
@@ -2378,7 +3192,7 @@
         <v>4.4360000000000002E-5</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11">
         <f>SourceData!G13</f>
         <v>2019</v>
@@ -2388,7 +3202,7 @@
         <v>4.5469000000000001E-5</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12">
         <f>SourceData!G14</f>
         <v>2020</v>
@@ -2398,7 +3212,7 @@
         <v>4.6578E-5</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13">
         <f>SourceData!G15</f>
         <v>2021</v>
@@ -2408,7 +3222,7 @@
         <v>4.6578E-5</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14">
         <f>SourceData!G16</f>
         <v>2022</v>
@@ -2418,7 +3232,7 @@
         <v>4.7686999999999999E-5</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15">
         <f>SourceData!G17</f>
         <v>2023</v>
@@ -2428,7 +3242,7 @@
         <v>4.8795999999999998E-5</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16">
         <f>SourceData!G18</f>
         <v>2024</v>
@@ -2438,7 +3252,7 @@
         <v>4.9905000000000004E-5</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17">
         <f>SourceData!G19</f>
         <v>2025</v>
@@ -2448,7 +3262,7 @@
         <v>5.1013999999999996E-5</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18">
         <f>SourceData!G20</f>
         <v>2026</v>
@@ -2458,7 +3272,7 @@
         <v>5.2122999999999995E-5</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19">
         <f>SourceData!G21</f>
         <v>2027</v>
@@ -2468,7 +3282,7 @@
         <v>5.3232000000000001E-5</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20">
         <f>SourceData!G22</f>
         <v>2028</v>
@@ -2478,7 +3292,7 @@
         <v>5.4341E-5</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21">
         <f>SourceData!G23</f>
         <v>2029</v>
@@ -2488,7 +3302,7 @@
         <v>5.4341E-5</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22">
         <f>SourceData!G24</f>
         <v>2030</v>
@@ -2498,7 +3312,7 @@
         <v>5.5450000000000006E-5</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23">
         <f>SourceData!G25</f>
         <v>2031</v>
@@ -2508,7 +3322,7 @@
         <v>5.6558999999999998E-5</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24">
         <f>SourceData!G26</f>
         <v>2032</v>
@@ -2518,7 +3332,7 @@
         <v>5.7667999999999997E-5</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25">
         <f>SourceData!G27</f>
         <v>2033</v>
@@ -2528,7 +3342,7 @@
         <v>5.8777000000000003E-5</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26">
         <f>SourceData!G28</f>
         <v>2034</v>
@@ -2538,7 +3352,7 @@
         <v>5.9885999999999995E-5</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27">
         <f>SourceData!G29</f>
         <v>2035</v>
@@ -2548,7 +3362,7 @@
         <v>6.0994999999999995E-5</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28">
         <f>SourceData!G30</f>
         <v>2036</v>
@@ -2558,7 +3372,7 @@
         <v>6.2104E-5</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29">
         <f>SourceData!G31</f>
         <v>2037</v>
@@ -2568,7 +3382,7 @@
         <v>6.3213000000000006E-5</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30">
         <f>SourceData!G32</f>
         <v>2038</v>
@@ -2578,7 +3392,7 @@
         <v>6.4321999999999998E-5</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31">
         <f>SourceData!G33</f>
         <v>2039</v>
@@ -2588,7 +3402,7 @@
         <v>6.5430999999999991E-5</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32">
         <f>SourceData!G34</f>
         <v>2040</v>
@@ -2598,7 +3412,7 @@
         <v>6.6539999999999997E-5</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33">
         <f>SourceData!G35</f>
         <v>2041</v>
@@ -2608,7 +3422,7 @@
         <v>6.7649000000000002E-5</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34">
         <f>SourceData!G36</f>
         <v>2042</v>
@@ -2618,7 +3432,7 @@
         <v>6.7649000000000002E-5</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35">
         <f>SourceData!G37</f>
         <v>2043</v>
@@ -2628,7 +3442,7 @@
         <v>6.8757999999999995E-5</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36">
         <f>SourceData!G38</f>
         <v>2044</v>
@@ -2638,7 +3452,7 @@
         <v>6.9867E-5</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37">
         <f>SourceData!G39</f>
         <v>2045</v>
@@ -2648,7 +3462,7 @@
         <v>7.0975999999999993E-5</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38">
         <f>SourceData!G40</f>
         <v>2046</v>
@@ -2658,7 +3472,7 @@
         <v>7.2084999999999998E-5</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39">
         <f>SourceData!G41</f>
         <v>2047</v>
@@ -2668,7 +3482,7 @@
         <v>7.3194000000000004E-5</v>
       </c>
     </row>
-    <row r="40" spans="1:2" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40">
         <f>SourceData!G42</f>
         <v>2048</v>
@@ -2678,7 +3492,7 @@
         <v>7.4302999999999997E-5</v>
       </c>
     </row>
-    <row r="41" spans="1:2" ht="14.45" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41">
         <f>SourceData!G43</f>
         <v>2049</v>
@@ -2688,7 +3502,7 @@
         <v>7.5412000000000002E-5</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42">
         <f>SourceData!G44</f>
         <v>2050</v>
@@ -2696,6 +3510,186 @@
       <c r="B42" s="12">
         <f>SourceData!I44</f>
         <v>7.6520999999999995E-5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" s="13">
+        <v>2051</v>
+      </c>
+      <c r="B43" s="12">
+        <f>SourceData!I45</f>
+        <v>7.6785057448410887E-5</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" s="13">
+        <v>2052</v>
+      </c>
+      <c r="B44" s="12">
+        <f>SourceData!I46</f>
+        <v>7.7779793920481984E-5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" s="13">
+        <v>2053</v>
+      </c>
+      <c r="B45" s="12">
+        <f>SourceData!I47</f>
+        <v>7.8843859092279862E-5</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" s="13">
+        <v>2054</v>
+      </c>
+      <c r="B46" s="12">
+        <f>SourceData!I48</f>
+        <v>7.9885387520073171E-5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="13">
+        <v>2055</v>
+      </c>
+      <c r="B47" s="12">
+        <f>SourceData!I49</f>
+        <v>8.0904750051638674E-5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" s="13">
+        <v>2056</v>
+      </c>
+      <c r="B48" s="12">
+        <f>SourceData!I50</f>
+        <v>8.1902647706332622E-5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" s="13">
+        <v>2057</v>
+      </c>
+      <c r="B49" s="12">
+        <f>SourceData!I51</f>
+        <v>8.2880238828853957E-5</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" s="13">
+        <v>2058</v>
+      </c>
+      <c r="B50" s="12">
+        <f>SourceData!I52</f>
+        <v>8.3888153693965412E-5</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" s="13">
+        <v>2059</v>
+      </c>
+      <c r="B51" s="12">
+        <f>SourceData!I53</f>
+        <v>8.4892180152976656E-5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52" s="13">
+        <v>2060</v>
+      </c>
+      <c r="B52" s="12">
+        <f>SourceData!I54</f>
+        <v>8.5921966198623651E-5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" s="13">
+        <v>2061</v>
+      </c>
+      <c r="B53" s="12">
+        <f>SourceData!I55</f>
+        <v>8.6948276429878846E-5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" s="13">
+        <v>2062</v>
+      </c>
+      <c r="B54" s="12">
+        <f>SourceData!I56</f>
+        <v>8.7976360715815845E-5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" s="13">
+        <v>2063</v>
+      </c>
+      <c r="B55" s="12">
+        <f>SourceData!I57</f>
+        <v>8.8955706998581889E-5</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" s="13">
+        <v>2064</v>
+      </c>
+      <c r="B56" s="12">
+        <f>SourceData!I58</f>
+        <v>8.994507332200543E-5</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" s="13">
+        <v>2065</v>
+      </c>
+      <c r="B57" s="12">
+        <f>SourceData!I59</f>
+        <v>9.0931133549412388E-5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" s="13">
+        <v>2066</v>
+      </c>
+      <c r="B58" s="12">
+        <f>SourceData!I60</f>
+        <v>9.1921167247548021E-5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" s="13">
+        <v>2067</v>
+      </c>
+      <c r="B59" s="12">
+        <f>SourceData!I61</f>
+        <v>9.2915986658587027E-5</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" s="13">
+        <v>2068</v>
+      </c>
+      <c r="B60" s="12">
+        <f>SourceData!I62</f>
+        <v>9.3915924582859314E-5</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" s="13">
+        <v>2069</v>
+      </c>
+      <c r="B61" s="12">
+        <f>SourceData!I63</f>
+        <v>9.4923079650955047E-5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" s="13">
+        <v>2070</v>
+      </c>
+      <c r="B62" s="12">
+        <f>SourceData!I64</f>
+        <v>9.5936643103957875E-5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>